<commit_message>
Team MSG-Titans4, links, user guide, diagrams
</commit_message>
<xml_diff>
--- a/backend/reports/rule_matrix.xlsx
+++ b/backend/reports/rule_matrix.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rule Matrix'!$A$1:$P$620</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'By Case'!$A$1:$P$117</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Rule Matrix'!$A$1:$P$630</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'By Case'!$A$1:$P$127</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P620"/>
+  <dimension ref="A1:P630"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -620,7 +620,7 @@
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>delayed_delivery_terms AND rule_001_evidence -- Standard domestic transit delay under 24 hours without perishable contents</t>
+          <t>delayed_delivery_terms -- Standard domestic transit delay under 24 hours without perishable contents</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
@@ -675,7 +675,7 @@
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>delayed_delivery_terms AND rule_001_evidence -- Standard domestic transit delay under 24 hours without perishable contents</t>
+          <t>delayed_delivery_terms -- Standard domestic transit delay under 24 hours without perishable contents</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -719,7 +719,7 @@
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>delayed_delivery_terms AND rule_001_evidence -- Standard domestic transit delay under 24 hours without perishable contents</t>
+          <t>delayed_delivery_terms -- Standard domestic transit delay under 24 hours without perishable contents</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -763,7 +763,7 @@
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>delayed_delivery_terms AND rule_001_evidence -- Standard domestic transit delay under 24 hours without perishable contents</t>
+          <t>delayed_delivery_terms -- Standard domestic transit delay under 24 hours without perishable contents</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -1501,7 +1501,7 @@
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>missed_delivery_attempt_terms AND rule_004_evidence -- First missed delivery attempt due to customer premises locked or phone unattended</t>
+          <t>missed_delivery_attempt_terms -- First missed delivery attempt due to customer premises locked or phone unattended</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -1556,7 +1556,7 @@
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>missed_delivery_attempt_terms AND rule_004_evidence -- First missed delivery attempt due to customer premises locked or phone unattended</t>
+          <t>missed_delivery_attempt_terms -- First missed delivery attempt due to customer premises locked or phone unattended</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
@@ -1600,7 +1600,7 @@
       <c r="C22" s="2" t="inlineStr"/>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>missed_delivery_attempt_terms AND rule_004_evidence -- First missed delivery attempt due to customer premises locked or phone unattended</t>
+          <t>missed_delivery_attempt_terms -- First missed delivery attempt due to customer premises locked or phone unattended</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr"/>
@@ -1644,7 +1644,7 @@
       <c r="C23" s="2" t="inlineStr"/>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>missed_delivery_attempt_terms AND rule_004_evidence -- First missed delivery attempt due to customer premises locked or phone unattended</t>
+          <t>missed_delivery_attempt_terms -- First missed delivery attempt due to customer premises locked or phone unattended</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr"/>
@@ -2034,7 +2034,11 @@
           <t>DOC-003-S4</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr"/>
       <c r="L30" s="2" t="inlineStr">
@@ -2322,7 +2326,7 @@
       <c r="C36" s="2" t="inlineStr"/>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>package_left_unattended_terms AND rule_007_evidence -- Package left on porch or with building guard with prior verbal consignee permission</t>
+          <t>package_left_unattended_terms -- Package left on porch or with building guard with prior verbal consignee permission</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr"/>
@@ -2375,7 +2379,7 @@
       <c r="C37" s="2" t="inlineStr"/>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>package_left_unattended_terms AND rule_007_evidence -- Package left on porch or with building guard with prior verbal consignee permission</t>
+          <t>package_left_unattended_terms -- Package left on porch or with building guard with prior verbal consignee permission</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
@@ -2419,7 +2423,7 @@
       <c r="C38" s="2" t="inlineStr"/>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>package_left_unattended_terms AND rule_007_evidence -- Package left on porch or with building guard with prior verbal consignee permission</t>
+          <t>package_left_unattended_terms -- Package left on porch or with building guard with prior verbal consignee permission</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr"/>
@@ -2463,7 +2467,7 @@
       <c r="C39" s="2" t="inlineStr"/>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>package_left_unattended_terms AND rule_007_evidence -- Package left on porch or with building guard with prior verbal consignee permission</t>
+          <t>package_left_unattended_terms -- Package left on porch or with building guard with prior verbal consignee permission</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr"/>
@@ -2538,7 +2542,11 @@
           <t>DOC-003-S3</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr"/>
@@ -3141,7 +3149,7 @@
       <c r="C52" s="2" t="inlineStr"/>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>wrong_route_dispatch_terms AND rule_010_evidence -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan</t>
+          <t>wrong_route_dispatch_terms -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr"/>
@@ -3196,7 +3204,7 @@
       <c r="C53" s="2" t="inlineStr"/>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>wrong_route_dispatch_terms AND rule_010_evidence -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan)</t>
+          <t>wrong_route_dispatch_terms -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan)</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr"/>
@@ -3240,7 +3248,7 @@
       <c r="C54" s="2" t="inlineStr"/>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>wrong_route_dispatch_terms AND rule_010_evidence -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan)</t>
+          <t>wrong_route_dispatch_terms -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan)</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr"/>
@@ -3284,7 +3292,7 @@
       <c r="C55" s="2" t="inlineStr"/>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>wrong_route_dispatch_terms AND rule_010_evidence -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan)</t>
+          <t>wrong_route_dispatch_terms -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan)</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr"/>
@@ -3988,7 +3996,11 @@
           <t>DOC-007-S1</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="2" t="inlineStr"/>
       <c r="L68" s="2" t="inlineStr">
@@ -4280,7 +4292,7 @@
       <c r="C74" s="2" t="inlineStr"/>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>lost_parcel_terms AND rule_014_evidence -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
+          <t>lost_parcel_terms -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -4340,7 +4352,7 @@
       <c r="C75" s="2" t="inlineStr"/>
       <c r="D75" s="2" t="inlineStr">
         <is>
-          <t>lost_parcel_terms AND rule_014_evidence -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
+          <t>lost_parcel_terms -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
         </is>
       </c>
       <c r="E75" s="2" t="inlineStr"/>
@@ -4395,7 +4407,7 @@
       <c r="C76" s="2" t="inlineStr"/>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>lost_parcel_terms AND rule_014_evidence -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
+          <t>lost_parcel_terms -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
         </is>
       </c>
       <c r="E76" s="2" t="inlineStr"/>
@@ -4439,7 +4451,7 @@
       <c r="C77" s="2" t="inlineStr"/>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>lost_parcel_terms AND rule_014_evidence -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
+          <t>lost_parcel_terms -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr"/>
@@ -4483,7 +4495,7 @@
       <c r="C78" s="2" t="inlineStr"/>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>lost_parcel_terms AND rule_014_evidence -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
+          <t>lost_parcel_terms -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr"/>
@@ -4873,7 +4885,11 @@
           <t>DOC-007-S2</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr"/>
+      <c r="I85" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J85" s="2" t="inlineStr"/>
       <c r="K85" s="2" t="inlineStr"/>
       <c r="L85" s="2" t="inlineStr">
@@ -5165,7 +5181,7 @@
       <c r="C91" s="2" t="inlineStr"/>
       <c r="D91" s="2" t="inlineStr">
         <is>
-          <t>partial_shipment_missing_terms AND rule_017_evidence -- Partial loss confirmed stolen from damaged outer master carton</t>
+          <t>partial_shipment_missing_terms -- Partial loss confirmed stolen from damaged outer master carton</t>
         </is>
       </c>
       <c r="E91" s="2" t="inlineStr">
@@ -5225,7 +5241,7 @@
       <c r="C92" s="2" t="inlineStr"/>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>partial_shipment_missing_terms AND rule_017_evidence -- Partial loss confirmed stolen from damaged outer master carton</t>
+          <t>partial_shipment_missing_terms -- Partial loss confirmed stolen from damaged outer master carton</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr"/>
@@ -5280,7 +5296,7 @@
       <c r="C93" s="2" t="inlineStr"/>
       <c r="D93" s="2" t="inlineStr">
         <is>
-          <t>partial_shipment_missing_terms AND rule_017_evidence -- Partial loss confirmed stolen from damaged outer master carton</t>
+          <t>partial_shipment_missing_terms -- Partial loss confirmed stolen from damaged outer master carton</t>
         </is>
       </c>
       <c r="E93" s="2" t="inlineStr"/>
@@ -5324,7 +5340,7 @@
       <c r="C94" s="2" t="inlineStr"/>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>partial_shipment_missing_terms AND rule_017_evidence -- Partial loss confirmed stolen from damaged outer master carton</t>
+          <t>partial_shipment_missing_terms -- Partial loss confirmed stolen from damaged outer master carton</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr"/>
@@ -5368,7 +5384,7 @@
       <c r="C95" s="2" t="inlineStr"/>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>partial_shipment_missing_terms AND rule_017_evidence -- Partial loss confirmed stolen from damaged outer master carton</t>
+          <t>partial_shipment_missing_terms -- Partial loss confirmed stolen from damaged outer master carton</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr"/>
@@ -5790,7 +5806,7 @@
       <c r="C103" s="2" t="inlineStr"/>
       <c r="D103" s="2" t="inlineStr">
         <is>
-          <t>damaged_parcel_terms AND rule_019_evidence -- Minor outer carton denting with internal goods completely undamaged</t>
+          <t>damaged_parcel_terms -- Minor outer carton denting with internal goods completely undamaged</t>
         </is>
       </c>
       <c r="E103" s="2" t="inlineStr"/>
@@ -5844,7 +5860,7 @@
       <c r="C104" s="2" t="inlineStr"/>
       <c r="D104" s="2" t="inlineStr">
         <is>
-          <t>damaged_parcel_terms AND rule_019_evidence -- Minor outer carton denting with internal goods completely undamaged</t>
+          <t>damaged_parcel_terms -- Minor outer carton denting with internal goods completely undamaged</t>
         </is>
       </c>
       <c r="E104" s="2" t="inlineStr"/>
@@ -5888,7 +5904,7 @@
       <c r="C105" s="2" t="inlineStr"/>
       <c r="D105" s="2" t="inlineStr">
         <is>
-          <t>damaged_parcel_terms AND rule_019_evidence -- Minor outer carton denting with internal goods completely undamaged</t>
+          <t>damaged_parcel_terms -- Minor outer carton denting with internal goods completely undamaged</t>
         </is>
       </c>
       <c r="E105" s="2" t="inlineStr"/>
@@ -5932,7 +5948,7 @@
       <c r="C106" s="2" t="inlineStr"/>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t>damaged_parcel_terms AND rule_019_evidence -- Minor outer carton denting with internal goods completely undamaged</t>
+          <t>damaged_parcel_terms -- Minor outer carton denting with internal goods completely undamaged</t>
         </is>
       </c>
       <c r="E106" s="2" t="inlineStr"/>
@@ -6007,7 +6023,11 @@
           <t>DOC-007-S2</t>
         </is>
       </c>
-      <c r="I107" s="2" t="inlineStr"/>
+      <c r="I107" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J107" s="2" t="inlineStr"/>
       <c r="K107" s="2" t="inlineStr"/>
       <c r="L107" s="2" t="inlineStr">
@@ -6925,7 +6945,7 @@
       <c r="C125" s="2" t="inlineStr"/>
       <c r="D125" s="2" t="inlineStr">
         <is>
-          <t>wrong_item_delivered_terms AND rule_023_evidence -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
+          <t>wrong_item_delivered_terms -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
         </is>
       </c>
       <c r="E125" s="2" t="inlineStr"/>
@@ -6980,7 +7000,7 @@
       <c r="C126" s="2" t="inlineStr"/>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t>wrong_item_delivered_terms AND rule_023_evidence -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
+          <t>wrong_item_delivered_terms -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
         </is>
       </c>
       <c r="E126" s="2" t="inlineStr"/>
@@ -7024,7 +7044,7 @@
       <c r="C127" s="2" t="inlineStr"/>
       <c r="D127" s="2" t="inlineStr">
         <is>
-          <t>wrong_item_delivered_terms AND rule_023_evidence -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
+          <t>wrong_item_delivered_terms -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
         </is>
       </c>
       <c r="E127" s="2" t="inlineStr"/>
@@ -7068,7 +7088,7 @@
       <c r="C128" s="2" t="inlineStr"/>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>wrong_item_delivered_terms AND rule_023_evidence -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
+          <t>wrong_item_delivered_terms -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
         </is>
       </c>
       <c r="E128" s="2" t="inlineStr"/>
@@ -7458,7 +7478,11 @@
           <t>DOC-009-S3</t>
         </is>
       </c>
-      <c r="I135" s="2" t="inlineStr"/>
+      <c r="I135" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J135" s="2" t="inlineStr"/>
       <c r="K135" s="2" t="inlineStr"/>
       <c r="L135" s="2" t="inlineStr"/>
@@ -7491,7 +7515,7 @@
       <c r="C136" s="2" t="inlineStr"/>
       <c r="D136" s="2" t="inlineStr">
         <is>
-          <t>tampered_packaging_terms AND rule_025_evidence -- Parcel received with broken security tape but all items accounted for and intact</t>
+          <t>tampered_packaging_terms -- Parcel received with broken security tape but all items accounted for and intact</t>
         </is>
       </c>
       <c r="E136" s="2" t="inlineStr"/>
@@ -7545,7 +7569,7 @@
       <c r="C137" s="2" t="inlineStr"/>
       <c r="D137" s="2" t="inlineStr">
         <is>
-          <t>tampered_packaging_terms AND rule_025_evidence -- Parcel received with broken security tape but all items accounted for and intact</t>
+          <t>tampered_packaging_terms -- Parcel received with broken security tape but all items accounted for and intact</t>
         </is>
       </c>
       <c r="E137" s="2" t="inlineStr"/>
@@ -7589,7 +7613,7 @@
       <c r="C138" s="2" t="inlineStr"/>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>tampered_packaging_terms AND rule_025_evidence -- Parcel received with broken security tape but all items accounted for and intact</t>
+          <t>tampered_packaging_terms -- Parcel received with broken security tape but all items accounted for and intact</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr"/>
@@ -7633,7 +7657,7 @@
       <c r="C139" s="2" t="inlineStr"/>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>tampered_packaging_terms AND rule_025_evidence -- Parcel received with broken security tape but all items accounted for and intact</t>
+          <t>tampered_packaging_terms -- Parcel received with broken security tape but all items accounted for and intact</t>
         </is>
       </c>
       <c r="E139" s="2" t="inlineStr"/>
@@ -8685,7 +8709,7 @@
       <c r="C159" s="2" t="inlineStr"/>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t>cod_amount_mismatch_terms AND rule_029_evidence -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
+          <t>cod_amount_mismatch_terms -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr"/>
@@ -8740,7 +8764,7 @@
       <c r="C160" s="2" t="inlineStr"/>
       <c r="D160" s="2" t="inlineStr">
         <is>
-          <t>cod_amount_mismatch_terms AND rule_029_evidence -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
+          <t>cod_amount_mismatch_terms -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
         </is>
       </c>
       <c r="E160" s="2" t="inlineStr"/>
@@ -8784,7 +8808,7 @@
       <c r="C161" s="2" t="inlineStr"/>
       <c r="D161" s="2" t="inlineStr">
         <is>
-          <t>cod_amount_mismatch_terms AND rule_029_evidence -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
+          <t>cod_amount_mismatch_terms -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
         </is>
       </c>
       <c r="E161" s="2" t="inlineStr"/>
@@ -8828,7 +8852,7 @@
       <c r="C162" s="2" t="inlineStr"/>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>cod_amount_mismatch_terms AND rule_029_evidence -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
+          <t>cod_amount_mismatch_terms -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr"/>
@@ -9255,7 +9279,7 @@
       <c r="C170" s="2" t="inlineStr"/>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>duplicate_charge_terms AND rule_031_evidence -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
+          <t>duplicate_charge_terms -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr"/>
@@ -9310,7 +9334,7 @@
       <c r="C171" s="2" t="inlineStr"/>
       <c r="D171" s="2" t="inlineStr">
         <is>
-          <t>duplicate_charge_terms AND rule_031_evidence -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
+          <t>duplicate_charge_terms -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
         </is>
       </c>
       <c r="E171" s="2" t="inlineStr"/>
@@ -9354,7 +9378,7 @@
       <c r="C172" s="2" t="inlineStr"/>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>duplicate_charge_terms AND rule_031_evidence -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
+          <t>duplicate_charge_terms -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr"/>
@@ -9398,7 +9422,7 @@
       <c r="C173" s="2" t="inlineStr"/>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>duplicate_charge_terms AND rule_031_evidence -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
+          <t>duplicate_charge_terms -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr"/>
@@ -10134,7 +10158,7 @@
       <c r="C187" s="2" t="inlineStr"/>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>incorrect_charge_terms AND rule_034_evidence -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,00</t>
+          <t>incorrect_charge_terms -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,00</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr"/>
@@ -10188,7 +10212,7 @@
       <c r="C188" s="2" t="inlineStr"/>
       <c r="D188" s="2" t="inlineStr">
         <is>
-          <t>incorrect_charge_terms AND rule_034_evidence -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,000)</t>
+          <t>incorrect_charge_terms -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,000)</t>
         </is>
       </c>
       <c r="E188" s="2" t="inlineStr"/>
@@ -10232,7 +10256,7 @@
       <c r="C189" s="2" t="inlineStr"/>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>incorrect_charge_terms AND rule_034_evidence -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,000)</t>
+          <t>incorrect_charge_terms -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,000)</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr"/>
@@ -10276,7 +10300,7 @@
       <c r="C190" s="2" t="inlineStr"/>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>incorrect_charge_terms AND rule_034_evidence -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,000)</t>
+          <t>incorrect_charge_terms -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,000)</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr"/>
@@ -11012,7 +11036,7 @@
       <c r="C204" s="2" t="inlineStr"/>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>cod_remittance_delay_terms AND rule_037_evidence -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
+          <t>cod_remittance_delay_terms -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr"/>
@@ -11065,7 +11089,7 @@
       <c r="C205" s="2" t="inlineStr"/>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>cod_remittance_delay_terms AND rule_037_evidence -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
+          <t>cod_remittance_delay_terms -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr"/>
@@ -11109,7 +11133,7 @@
       <c r="C206" s="2" t="inlineStr"/>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>cod_remittance_delay_terms AND rule_037_evidence -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
+          <t>cod_remittance_delay_terms -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr"/>
@@ -11153,7 +11177,7 @@
       <c r="C207" s="2" t="inlineStr"/>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>cod_remittance_delay_terms AND rule_037_evidence -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
+          <t>cod_remittance_delay_terms -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr"/>
@@ -11895,7 +11919,7 @@
       <c r="C221" s="2" t="inlineStr"/>
       <c r="D221" s="2" t="inlineStr">
         <is>
-          <t>refund_not_processed_terms AND rule_040_evidence -- Customer refund requested within 7-day policy window, all documentation verified</t>
+          <t>refund_not_processed_terms -- Customer refund requested within 7-day policy window, all documentation verified</t>
         </is>
       </c>
       <c r="E221" s="2" t="inlineStr"/>
@@ -11950,7 +11974,7 @@
       <c r="C222" s="2" t="inlineStr"/>
       <c r="D222" s="2" t="inlineStr">
         <is>
-          <t>refund_not_processed_terms AND rule_040_evidence -- Customer refund requested within 7-day policy window, all documentation verified</t>
+          <t>refund_not_processed_terms -- Customer refund requested within 7-day policy window, all documentation verified</t>
         </is>
       </c>
       <c r="E222" s="2" t="inlineStr"/>
@@ -11994,7 +12018,7 @@
       <c r="C223" s="2" t="inlineStr"/>
       <c r="D223" s="2" t="inlineStr">
         <is>
-          <t>refund_not_processed_terms AND rule_040_evidence -- Customer refund requested within 7-day policy window, all documentation verified</t>
+          <t>refund_not_processed_terms -- Customer refund requested within 7-day policy window, all documentation verified</t>
         </is>
       </c>
       <c r="E223" s="2" t="inlineStr"/>
@@ -12038,7 +12062,7 @@
       <c r="C224" s="2" t="inlineStr"/>
       <c r="D224" s="2" t="inlineStr">
         <is>
-          <t>refund_not_processed_terms AND rule_040_evidence -- Customer refund requested within 7-day policy window, all documentation verified</t>
+          <t>refund_not_processed_terms -- Customer refund requested within 7-day policy window, all documentation verified</t>
         </is>
       </c>
       <c r="E224" s="2" t="inlineStr"/>
@@ -12776,7 +12800,7 @@
       <c r="C238" s="2" t="inlineStr"/>
       <c r="D238" s="2" t="inlineStr">
         <is>
-          <t>refund_delay_terms AND rule_043_evidence -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
+          <t>refund_delay_terms -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
         </is>
       </c>
       <c r="E238" s="2" t="inlineStr"/>
@@ -12830,7 +12854,7 @@
       <c r="C239" s="2" t="inlineStr"/>
       <c r="D239" s="2" t="inlineStr">
         <is>
-          <t>refund_delay_terms AND rule_043_evidence -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
+          <t>refund_delay_terms -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
         </is>
       </c>
       <c r="E239" s="2" t="inlineStr"/>
@@ -12874,7 +12898,7 @@
       <c r="C240" s="2" t="inlineStr"/>
       <c r="D240" s="2" t="inlineStr">
         <is>
-          <t>refund_delay_terms AND rule_043_evidence -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
+          <t>refund_delay_terms -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
         </is>
       </c>
       <c r="E240" s="2" t="inlineStr"/>
@@ -12918,7 +12942,7 @@
       <c r="C241" s="2" t="inlineStr"/>
       <c r="D241" s="2" t="inlineStr">
         <is>
-          <t>refund_delay_terms AND rule_043_evidence -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
+          <t>refund_delay_terms -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
         </is>
       </c>
       <c r="E241" s="2" t="inlineStr"/>
@@ -13594,7 +13618,7 @@
       <c r="C254" s="2" t="inlineStr"/>
       <c r="D254" s="2" t="inlineStr">
         <is>
-          <t>rto_processing_delay_terms AND rule_046_evidence -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
+          <t>rto_processing_delay_terms -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
         </is>
       </c>
       <c r="E254" s="2" t="inlineStr"/>
@@ -13647,7 +13671,7 @@
       <c r="C255" s="2" t="inlineStr"/>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t>rto_processing_delay_terms AND rule_046_evidence -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
+          <t>rto_processing_delay_terms -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
         </is>
       </c>
       <c r="E255" s="2" t="inlineStr"/>
@@ -13691,7 +13715,7 @@
       <c r="C256" s="2" t="inlineStr"/>
       <c r="D256" s="2" t="inlineStr">
         <is>
-          <t>rto_processing_delay_terms AND rule_046_evidence -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
+          <t>rto_processing_delay_terms -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
         </is>
       </c>
       <c r="E256" s="2" t="inlineStr"/>
@@ -13735,7 +13759,7 @@
       <c r="C257" s="2" t="inlineStr"/>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t>rto_processing_delay_terms AND rule_046_evidence -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
+          <t>rto_processing_delay_terms -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
         </is>
       </c>
       <c r="E257" s="2" t="inlineStr"/>
@@ -14472,7 +14496,7 @@
       <c r="C271" s="2" t="inlineStr"/>
       <c r="D271" s="2" t="inlineStr">
         <is>
-          <t>account_locked_terms AND rule_049_evidence -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
+          <t>account_locked_terms -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
         </is>
       </c>
       <c r="E271" s="2" t="inlineStr"/>
@@ -14527,7 +14551,7 @@
       <c r="C272" s="2" t="inlineStr"/>
       <c r="D272" s="2" t="inlineStr">
         <is>
-          <t>account_locked_terms AND rule_049_evidence -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
+          <t>account_locked_terms -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
         </is>
       </c>
       <c r="E272" s="2" t="inlineStr"/>
@@ -14571,7 +14595,7 @@
       <c r="C273" s="2" t="inlineStr"/>
       <c r="D273" s="2" t="inlineStr">
         <is>
-          <t>account_locked_terms AND rule_049_evidence -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
+          <t>account_locked_terms -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
         </is>
       </c>
       <c r="E273" s="2" t="inlineStr"/>
@@ -14615,7 +14639,7 @@
       <c r="C274" s="2" t="inlineStr"/>
       <c r="D274" s="2" t="inlineStr">
         <is>
-          <t>account_locked_terms AND rule_049_evidence -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
+          <t>account_locked_terms -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
         </is>
       </c>
       <c r="E274" s="2" t="inlineStr"/>
@@ -15355,7 +15379,7 @@
       <c r="C288" s="2" t="inlineStr"/>
       <c r="D288" s="2" t="inlineStr">
         <is>
-          <t>unauthorized_account_access_terms AND rule_052_evidence -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
+          <t>unauthorized_account_access_terms -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
         </is>
       </c>
       <c r="E288" s="2" t="inlineStr">
@@ -15415,7 +15439,7 @@
       <c r="C289" s="2" t="inlineStr"/>
       <c r="D289" s="2" t="inlineStr">
         <is>
-          <t>unauthorized_account_access_terms AND rule_052_evidence -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
+          <t>unauthorized_account_access_terms -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
         </is>
       </c>
       <c r="E289" s="2" t="inlineStr"/>
@@ -15469,7 +15493,7 @@
       <c r="C290" s="2" t="inlineStr"/>
       <c r="D290" s="2" t="inlineStr">
         <is>
-          <t>unauthorized_account_access_terms AND rule_052_evidence -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
+          <t>unauthorized_account_access_terms -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
         </is>
       </c>
       <c r="E290" s="2" t="inlineStr"/>
@@ -15513,7 +15537,7 @@
       <c r="C291" s="2" t="inlineStr"/>
       <c r="D291" s="2" t="inlineStr">
         <is>
-          <t>unauthorized_account_access_terms AND rule_052_evidence -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
+          <t>unauthorized_account_access_terms -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
         </is>
       </c>
       <c r="E291" s="2" t="inlineStr"/>
@@ -15557,7 +15581,7 @@
       <c r="C292" s="2" t="inlineStr"/>
       <c r="D292" s="2" t="inlineStr">
         <is>
-          <t>unauthorized_account_access_terms AND rule_052_evidence -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
+          <t>unauthorized_account_access_terms -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
         </is>
       </c>
       <c r="E292" s="2" t="inlineStr"/>
@@ -16294,7 +16318,7 @@
       <c r="C306" s="2" t="inlineStr"/>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t>merchant_profile_update_terms AND rule_055_evidence -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
+          <t>merchant_profile_update_terms -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr"/>
@@ -16348,7 +16372,7 @@
       <c r="C307" s="2" t="inlineStr"/>
       <c r="D307" s="2" t="inlineStr">
         <is>
-          <t>merchant_profile_update_terms AND rule_055_evidence -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
+          <t>merchant_profile_update_terms -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
         </is>
       </c>
       <c r="E307" s="2" t="inlineStr"/>
@@ -16392,7 +16416,7 @@
       <c r="C308" s="2" t="inlineStr"/>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>merchant_profile_update_terms AND rule_055_evidence -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
+          <t>merchant_profile_update_terms -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr"/>
@@ -16436,7 +16460,7 @@
       <c r="C309" s="2" t="inlineStr"/>
       <c r="D309" s="2" t="inlineStr">
         <is>
-          <t>merchant_profile_update_terms AND rule_055_evidence -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
+          <t>merchant_profile_update_terms -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
         </is>
       </c>
       <c r="E309" s="2" t="inlineStr"/>
@@ -16511,7 +16535,11 @@
           <t>DOC-021-S1</t>
         </is>
       </c>
-      <c r="I310" s="2" t="inlineStr"/>
+      <c r="I310" s="2" t="inlineStr">
+        <is>
+          <t>COMPLIANCE_REVIEW</t>
+        </is>
+      </c>
       <c r="J310" s="2" t="inlineStr"/>
       <c r="K310" s="2" t="inlineStr"/>
       <c r="L310" s="2" t="inlineStr">
@@ -17113,7 +17141,7 @@
       <c r="C322" s="2" t="inlineStr"/>
       <c r="D322" s="2" t="inlineStr">
         <is>
-          <t>tracking_not_updating_terms AND rule_058_evidence -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
+          <t>tracking_not_updating_terms -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
         </is>
       </c>
       <c r="E322" s="2" t="inlineStr"/>
@@ -17167,7 +17195,7 @@
       <c r="C323" s="2" t="inlineStr"/>
       <c r="D323" s="2" t="inlineStr">
         <is>
-          <t>tracking_not_updating_terms AND rule_058_evidence -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
+          <t>tracking_not_updating_terms -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
         </is>
       </c>
       <c r="E323" s="2" t="inlineStr"/>
@@ -17211,7 +17239,7 @@
       <c r="C324" s="2" t="inlineStr"/>
       <c r="D324" s="2" t="inlineStr">
         <is>
-          <t>tracking_not_updating_terms AND rule_058_evidence -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
+          <t>tracking_not_updating_terms -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
         </is>
       </c>
       <c r="E324" s="2" t="inlineStr"/>
@@ -17255,7 +17283,7 @@
       <c r="C325" s="2" t="inlineStr"/>
       <c r="D325" s="2" t="inlineStr">
         <is>
-          <t>tracking_not_updating_terms AND rule_058_evidence -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
+          <t>tracking_not_updating_terms -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
         </is>
       </c>
       <c r="E325" s="2" t="inlineStr"/>
@@ -17991,7 +18019,7 @@
       <c r="C339" s="2" t="inlineStr"/>
       <c r="D339" s="2" t="inlineStr">
         <is>
-          <t>app_crash_terms AND rule_061_evidence -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
+          <t>app_crash_terms -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
         </is>
       </c>
       <c r="E339" s="2" t="inlineStr"/>
@@ -18045,7 +18073,7 @@
       <c r="C340" s="2" t="inlineStr"/>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t>app_crash_terms AND rule_061_evidence -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
+          <t>app_crash_terms -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr"/>
@@ -18089,7 +18117,7 @@
       <c r="C341" s="2" t="inlineStr"/>
       <c r="D341" s="2" t="inlineStr">
         <is>
-          <t>app_crash_terms AND rule_061_evidence -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
+          <t>app_crash_terms -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
         </is>
       </c>
       <c r="E341" s="2" t="inlineStr"/>
@@ -18133,7 +18161,7 @@
       <c r="C342" s="2" t="inlineStr"/>
       <c r="D342" s="2" t="inlineStr">
         <is>
-          <t>app_crash_terms AND rule_061_evidence -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
+          <t>app_crash_terms -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
         </is>
       </c>
       <c r="E342" s="2" t="inlineStr"/>
@@ -18522,7 +18550,11 @@
           <t>DOC-023-S2</t>
         </is>
       </c>
-      <c r="I349" s="2" t="inlineStr"/>
+      <c r="I349" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J349" s="2" t="inlineStr"/>
       <c r="K349" s="2" t="inlineStr"/>
       <c r="L349" s="2" t="inlineStr">
@@ -18809,7 +18841,7 @@
       <c r="C355" s="2" t="inlineStr"/>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t>api_webhook_failure_terms AND rule_064_evidence -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
+          <t>api_webhook_failure_terms -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr"/>
@@ -18863,7 +18895,7 @@
       <c r="C356" s="2" t="inlineStr"/>
       <c r="D356" s="2" t="inlineStr">
         <is>
-          <t>api_webhook_failure_terms AND rule_064_evidence -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
+          <t>api_webhook_failure_terms -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
         </is>
       </c>
       <c r="E356" s="2" t="inlineStr"/>
@@ -18907,7 +18939,7 @@
       <c r="C357" s="2" t="inlineStr"/>
       <c r="D357" s="2" t="inlineStr">
         <is>
-          <t>api_webhook_failure_terms AND rule_064_evidence -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
+          <t>api_webhook_failure_terms -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
         </is>
       </c>
       <c r="E357" s="2" t="inlineStr"/>
@@ -18951,7 +18983,7 @@
       <c r="C358" s="2" t="inlineStr"/>
       <c r="D358" s="2" t="inlineStr">
         <is>
-          <t>api_webhook_failure_terms AND rule_064_evidence -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
+          <t>api_webhook_failure_terms -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
         </is>
       </c>
       <c r="E358" s="2" t="inlineStr"/>
@@ -19026,7 +19058,11 @@
           <t>DOC-023-S2</t>
         </is>
       </c>
-      <c r="I359" s="2" t="inlineStr"/>
+      <c r="I359" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J359" s="2" t="inlineStr"/>
       <c r="K359" s="2" t="inlineStr"/>
       <c r="L359" s="2" t="inlineStr">
@@ -19594,7 +19630,11 @@
           <t>DOC-020-S1</t>
         </is>
       </c>
-      <c r="I370" s="2" t="inlineStr"/>
+      <c r="I370" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J370" s="2" t="inlineStr"/>
       <c r="K370" s="2" t="inlineStr"/>
       <c r="L370" s="2" t="inlineStr">
@@ -19631,7 +19671,7 @@
       <c r="C371" s="2" t="inlineStr"/>
       <c r="D371" s="2" t="inlineStr">
         <is>
-          <t>rude_rider_driver_behavior_terms AND rule_067_evidence -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
+          <t>rude_rider_driver_behavior_terms -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
         </is>
       </c>
       <c r="E371" s="2" t="inlineStr"/>
@@ -19686,7 +19726,7 @@
       <c r="C372" s="2" t="inlineStr"/>
       <c r="D372" s="2" t="inlineStr">
         <is>
-          <t>rude_rider_driver_behavior_terms AND rule_067_evidence -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
+          <t>rude_rider_driver_behavior_terms -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
         </is>
       </c>
       <c r="E372" s="2" t="inlineStr"/>
@@ -19730,7 +19770,7 @@
       <c r="C373" s="2" t="inlineStr"/>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t>rude_rider_driver_behavior_terms AND rule_067_evidence -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
+          <t>rude_rider_driver_behavior_terms -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
         </is>
       </c>
       <c r="E373" s="2" t="inlineStr"/>
@@ -19774,7 +19814,7 @@
       <c r="C374" s="2" t="inlineStr"/>
       <c r="D374" s="2" t="inlineStr">
         <is>
-          <t>rude_rider_driver_behavior_terms AND rule_067_evidence -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
+          <t>rude_rider_driver_behavior_terms -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
         </is>
       </c>
       <c r="E374" s="2" t="inlineStr"/>
@@ -20478,7 +20518,11 @@
           <t>DOC-021-S2</t>
         </is>
       </c>
-      <c r="I387" s="2" t="inlineStr"/>
+      <c r="I387" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J387" s="2" t="inlineStr"/>
       <c r="K387" s="2" t="inlineStr"/>
       <c r="L387" s="2" t="inlineStr"/>
@@ -20511,7 +20555,7 @@
       <c r="C388" s="2" t="inlineStr"/>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>rider_demanding_cash_tip_terms AND rule_070_evidence -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and rece</t>
+          <t>rider_demanding_cash_tip_terms -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and rece</t>
         </is>
       </c>
       <c r="E388" s="2" t="inlineStr"/>
@@ -20565,7 +20609,7 @@
       <c r="C389" s="2" t="inlineStr"/>
       <c r="D389" s="2" t="inlineStr">
         <is>
-          <t>rider_demanding_cash_tip_terms AND rule_070_evidence -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and received parcel</t>
+          <t>rider_demanding_cash_tip_terms -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and received parcel</t>
         </is>
       </c>
       <c r="E389" s="2" t="inlineStr"/>
@@ -20609,7 +20653,7 @@
       <c r="C390" s="2" t="inlineStr"/>
       <c r="D390" s="2" t="inlineStr">
         <is>
-          <t>rider_demanding_cash_tip_terms AND rule_070_evidence -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and received parcel</t>
+          <t>rider_demanding_cash_tip_terms -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and received parcel</t>
         </is>
       </c>
       <c r="E390" s="2" t="inlineStr"/>
@@ -20653,7 +20697,7 @@
       <c r="C391" s="2" t="inlineStr"/>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t>rider_demanding_cash_tip_terms AND rule_070_evidence -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and received parcel</t>
+          <t>rider_demanding_cash_tip_terms -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and received parcel</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr"/>
@@ -21390,7 +21434,7 @@
       <c r="C405" s="2" t="inlineStr"/>
       <c r="D405" s="2" t="inlineStr">
         <is>
-          <t>warranty_claim_denied_terms AND rule_073_evidence -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
+          <t>warranty_claim_denied_terms -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
         </is>
       </c>
       <c r="E405" s="2" t="inlineStr"/>
@@ -21445,7 +21489,7 @@
       <c r="C406" s="2" t="inlineStr"/>
       <c r="D406" s="2" t="inlineStr">
         <is>
-          <t>warranty_claim_denied_terms AND rule_073_evidence -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
+          <t>warranty_claim_denied_terms -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
         </is>
       </c>
       <c r="E406" s="2" t="inlineStr"/>
@@ -21489,7 +21533,7 @@
       <c r="C407" s="2" t="inlineStr"/>
       <c r="D407" s="2" t="inlineStr">
         <is>
-          <t>warranty_claim_denied_terms AND rule_073_evidence -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
+          <t>warranty_claim_denied_terms -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
         </is>
       </c>
       <c r="E407" s="2" t="inlineStr"/>
@@ -21533,7 +21577,7 @@
       <c r="C408" s="2" t="inlineStr"/>
       <c r="D408" s="2" t="inlineStr">
         <is>
-          <t>warranty_claim_denied_terms AND rule_073_evidence -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
+          <t>warranty_claim_denied_terms -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
         </is>
       </c>
       <c r="E408" s="2" t="inlineStr"/>
@@ -22269,7 +22313,7 @@
       <c r="C422" s="2" t="inlineStr"/>
       <c r="D422" s="2" t="inlineStr">
         <is>
-          <t>insurance_payout_delay_terms AND rule_076_evidence -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
+          <t>insurance_payout_delay_terms -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
         </is>
       </c>
       <c r="E422" s="2" t="inlineStr"/>
@@ -22322,7 +22366,7 @@
       <c r="C423" s="2" t="inlineStr"/>
       <c r="D423" s="2" t="inlineStr">
         <is>
-          <t>insurance_payout_delay_terms AND rule_076_evidence -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
+          <t>insurance_payout_delay_terms -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
         </is>
       </c>
       <c r="E423" s="2" t="inlineStr"/>
@@ -22366,7 +22410,7 @@
       <c r="C424" s="2" t="inlineStr"/>
       <c r="D424" s="2" t="inlineStr">
         <is>
-          <t>insurance_payout_delay_terms AND rule_076_evidence -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
+          <t>insurance_payout_delay_terms -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
         </is>
       </c>
       <c r="E424" s="2" t="inlineStr"/>
@@ -22410,7 +22454,7 @@
       <c r="C425" s="2" t="inlineStr"/>
       <c r="D425" s="2" t="inlineStr">
         <is>
-          <t>insurance_payout_delay_terms AND rule_076_evidence -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
+          <t>insurance_payout_delay_terms -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
         </is>
       </c>
       <c r="E425" s="2" t="inlineStr"/>
@@ -23150,7 +23194,7 @@
       <c r="C439" s="2" t="inlineStr"/>
       <c r="D439" s="2" t="inlineStr">
         <is>
-          <t>data_privacy_breach_terms AND rule_079_evidence -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
+          <t>data_privacy_breach_terms -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
         </is>
       </c>
       <c r="E439" s="2" t="inlineStr">
@@ -23210,7 +23254,7 @@
       <c r="C440" s="2" t="inlineStr"/>
       <c r="D440" s="2" t="inlineStr">
         <is>
-          <t>data_privacy_breach_terms AND rule_079_evidence -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
+          <t>data_privacy_breach_terms -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
         </is>
       </c>
       <c r="E440" s="2" t="inlineStr"/>
@@ -23265,7 +23309,7 @@
       <c r="C441" s="2" t="inlineStr"/>
       <c r="D441" s="2" t="inlineStr">
         <is>
-          <t>data_privacy_breach_terms AND rule_079_evidence -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
+          <t>data_privacy_breach_terms -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
         </is>
       </c>
       <c r="E441" s="2" t="inlineStr"/>
@@ -23309,7 +23353,7 @@
       <c r="C442" s="2" t="inlineStr"/>
       <c r="D442" s="2" t="inlineStr">
         <is>
-          <t>data_privacy_breach_terms AND rule_079_evidence -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
+          <t>data_privacy_breach_terms -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
         </is>
       </c>
       <c r="E442" s="2" t="inlineStr"/>
@@ -23353,7 +23397,7 @@
       <c r="C443" s="2" t="inlineStr"/>
       <c r="D443" s="2" t="inlineStr">
         <is>
-          <t>data_privacy_breach_terms AND rule_079_evidence -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
+          <t>data_privacy_breach_terms -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
         </is>
       </c>
       <c r="E443" s="2" t="inlineStr"/>
@@ -23743,7 +23787,11 @@
           <t>DOC-015-S3</t>
         </is>
       </c>
-      <c r="I450" s="2" t="inlineStr"/>
+      <c r="I450" s="2" t="inlineStr">
+        <is>
+          <t>COMPLIANCE_REVIEW</t>
+        </is>
+      </c>
       <c r="J450" s="2" t="inlineStr"/>
       <c r="K450" s="2" t="inlineStr"/>
       <c r="L450" s="2" t="inlineStr"/>
@@ -24026,7 +24074,7 @@
       <c r="C456" s="2" t="inlineStr"/>
       <c r="D456" s="2" t="inlineStr">
         <is>
-          <t>unsolicited_marketing_sms_terms AND rule_082_evidence -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
+          <t>unsolicited_marketing_sms_terms -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
         </is>
       </c>
       <c r="E456" s="2" t="inlineStr"/>
@@ -24079,7 +24127,7 @@
       <c r="C457" s="2" t="inlineStr"/>
       <c r="D457" s="2" t="inlineStr">
         <is>
-          <t>unsolicited_marketing_sms_terms AND rule_082_evidence -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
+          <t>unsolicited_marketing_sms_terms -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
         </is>
       </c>
       <c r="E457" s="2" t="inlineStr"/>
@@ -24123,7 +24171,7 @@
       <c r="C458" s="2" t="inlineStr"/>
       <c r="D458" s="2" t="inlineStr">
         <is>
-          <t>unsolicited_marketing_sms_terms AND rule_082_evidence -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
+          <t>unsolicited_marketing_sms_terms -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
         </is>
       </c>
       <c r="E458" s="2" t="inlineStr"/>
@@ -24167,7 +24215,7 @@
       <c r="C459" s="2" t="inlineStr"/>
       <c r="D459" s="2" t="inlineStr">
         <is>
-          <t>unsolicited_marketing_sms_terms AND rule_082_evidence -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
+          <t>unsolicited_marketing_sms_terms -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
         </is>
       </c>
       <c r="E459" s="2" t="inlineStr"/>
@@ -24903,7 +24951,7 @@
       <c r="C473" s="2" t="inlineStr"/>
       <c r="D473" s="2" t="inlineStr">
         <is>
-          <t>reckless_driving_safety_risk_terms AND rule_085_evidence -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
+          <t>reckless_driving_safety_risk_terms -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
         </is>
       </c>
       <c r="E473" s="2" t="inlineStr">
@@ -24963,7 +25011,7 @@
       <c r="C474" s="2" t="inlineStr"/>
       <c r="D474" s="2" t="inlineStr">
         <is>
-          <t>reckless_driving_safety_risk_terms AND rule_085_evidence -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
+          <t>reckless_driving_safety_risk_terms -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
         </is>
       </c>
       <c r="E474" s="2" t="inlineStr"/>
@@ -25017,7 +25065,7 @@
       <c r="C475" s="2" t="inlineStr"/>
       <c r="D475" s="2" t="inlineStr">
         <is>
-          <t>reckless_driving_safety_risk_terms AND rule_085_evidence -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
+          <t>reckless_driving_safety_risk_terms -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
         </is>
       </c>
       <c r="E475" s="2" t="inlineStr"/>
@@ -25061,7 +25109,7 @@
       <c r="C476" s="2" t="inlineStr"/>
       <c r="D476" s="2" t="inlineStr">
         <is>
-          <t>reckless_driving_safety_risk_terms AND rule_085_evidence -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
+          <t>reckless_driving_safety_risk_terms -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
         </is>
       </c>
       <c r="E476" s="2" t="inlineStr"/>
@@ -25105,7 +25153,7 @@
       <c r="C477" s="2" t="inlineStr"/>
       <c r="D477" s="2" t="inlineStr">
         <is>
-          <t>reckless_driving_safety_risk_terms AND rule_085_evidence -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
+          <t>reckless_driving_safety_risk_terms -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
         </is>
       </c>
       <c r="E477" s="2" t="inlineStr"/>
@@ -25810,7 +25858,11 @@
           <t>DOC-025-S2</t>
         </is>
       </c>
-      <c r="I490" s="2" t="inlineStr"/>
+      <c r="I490" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J490" s="2" t="inlineStr"/>
       <c r="K490" s="2" t="inlineStr"/>
       <c r="L490" s="2" t="inlineStr">
@@ -25847,7 +25899,7 @@
       <c r="C491" s="2" t="inlineStr"/>
       <c r="D491" s="2" t="inlineStr">
         <is>
-          <t>hazardous_material_mishandling_terms AND rule_088_evidence -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
+          <t>hazardous_material_mishandling_terms -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
         </is>
       </c>
       <c r="E491" s="2" t="inlineStr"/>
@@ -25902,7 +25954,7 @@
       <c r="C492" s="2" t="inlineStr"/>
       <c r="D492" s="2" t="inlineStr">
         <is>
-          <t>hazardous_material_mishandling_terms AND rule_088_evidence -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
+          <t>hazardous_material_mishandling_terms -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
         </is>
       </c>
       <c r="E492" s="2" t="inlineStr"/>
@@ -25946,7 +25998,7 @@
       <c r="C493" s="2" t="inlineStr"/>
       <c r="D493" s="2" t="inlineStr">
         <is>
-          <t>hazardous_material_mishandling_terms AND rule_088_evidence -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
+          <t>hazardous_material_mishandling_terms -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
         </is>
       </c>
       <c r="E493" s="2" t="inlineStr"/>
@@ -25990,7 +26042,7 @@
       <c r="C494" s="2" t="inlineStr"/>
       <c r="D494" s="2" t="inlineStr">
         <is>
-          <t>hazardous_material_mishandling_terms AND rule_088_evidence -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
+          <t>hazardous_material_mishandling_terms -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
         </is>
       </c>
       <c r="E494" s="2" t="inlineStr"/>
@@ -26727,7 +26779,7 @@
       <c r="C508" s="2" t="inlineStr"/>
       <c r="D508" s="2" t="inlineStr">
         <is>
-          <t>missing_customs_documents_terms AND rule_091_evidence -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on</t>
+          <t>missing_customs_documents_terms -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on</t>
         </is>
       </c>
       <c r="E508" s="2" t="inlineStr"/>
@@ -26781,7 +26833,7 @@
       <c r="C509" s="2" t="inlineStr"/>
       <c r="D509" s="2" t="inlineStr">
         <is>
-          <t>missing_customs_documents_terms AND rule_091_evidence -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on file</t>
+          <t>missing_customs_documents_terms -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on file</t>
         </is>
       </c>
       <c r="E509" s="2" t="inlineStr"/>
@@ -26825,7 +26877,7 @@
       <c r="C510" s="2" t="inlineStr"/>
       <c r="D510" s="2" t="inlineStr">
         <is>
-          <t>missing_customs_documents_terms AND rule_091_evidence -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on file</t>
+          <t>missing_customs_documents_terms -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on file</t>
         </is>
       </c>
       <c r="E510" s="2" t="inlineStr"/>
@@ -26869,7 +26921,7 @@
       <c r="C511" s="2" t="inlineStr"/>
       <c r="D511" s="2" t="inlineStr">
         <is>
-          <t>missing_customs_documents_terms AND rule_091_evidence -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on file</t>
+          <t>missing_customs_documents_terms -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on file</t>
         </is>
       </c>
       <c r="E511" s="2" t="inlineStr"/>
@@ -27606,7 +27658,7 @@
       <c r="C525" s="2" t="inlineStr"/>
       <c r="D525" s="2" t="inlineStr">
         <is>
-          <t>regulatory_impoundment_hold_terms AND rule_094_evidence -- Consignment held for routine random provincial excise vehicle weight and document check</t>
+          <t>regulatory_impoundment_hold_terms -- Consignment held for routine random provincial excise vehicle weight and document check</t>
         </is>
       </c>
       <c r="E525" s="2" t="inlineStr"/>
@@ -27660,7 +27712,7 @@
       <c r="C526" s="2" t="inlineStr"/>
       <c r="D526" s="2" t="inlineStr">
         <is>
-          <t>regulatory_impoundment_hold_terms AND rule_094_evidence -- Consignment held for routine random provincial excise vehicle weight and document check</t>
+          <t>regulatory_impoundment_hold_terms -- Consignment held for routine random provincial excise vehicle weight and document check</t>
         </is>
       </c>
       <c r="E526" s="2" t="inlineStr"/>
@@ -27704,7 +27756,7 @@
       <c r="C527" s="2" t="inlineStr"/>
       <c r="D527" s="2" t="inlineStr">
         <is>
-          <t>regulatory_impoundment_hold_terms AND rule_094_evidence -- Consignment held for routine random provincial excise vehicle weight and document check</t>
+          <t>regulatory_impoundment_hold_terms -- Consignment held for routine random provincial excise vehicle weight and document check</t>
         </is>
       </c>
       <c r="E527" s="2" t="inlineStr"/>
@@ -27748,7 +27800,7 @@
       <c r="C528" s="2" t="inlineStr"/>
       <c r="D528" s="2" t="inlineStr">
         <is>
-          <t>regulatory_impoundment_hold_terms AND rule_094_evidence -- Consignment held for routine random provincial excise vehicle weight and document check</t>
+          <t>regulatory_impoundment_hold_terms -- Consignment held for routine random provincial excise vehicle weight and document check</t>
         </is>
       </c>
       <c r="E528" s="2" t="inlineStr"/>
@@ -28484,7 +28536,7 @@
       <c r="C542" s="2" t="inlineStr"/>
       <c r="D542" s="2" t="inlineStr">
         <is>
-          <t>subscription_contract_renewal_terms AND rule_097_evidence -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
+          <t>subscription_contract_renewal_terms -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
         </is>
       </c>
       <c r="E542" s="2" t="inlineStr"/>
@@ -28538,7 +28590,7 @@
       <c r="C543" s="2" t="inlineStr"/>
       <c r="D543" s="2" t="inlineStr">
         <is>
-          <t>subscription_contract_renewal_terms AND rule_097_evidence -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
+          <t>subscription_contract_renewal_terms -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
         </is>
       </c>
       <c r="E543" s="2" t="inlineStr"/>
@@ -28582,7 +28634,7 @@
       <c r="C544" s="2" t="inlineStr"/>
       <c r="D544" s="2" t="inlineStr">
         <is>
-          <t>subscription_contract_renewal_terms AND rule_097_evidence -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
+          <t>subscription_contract_renewal_terms -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
         </is>
       </c>
       <c r="E544" s="2" t="inlineStr"/>
@@ -28626,7 +28678,7 @@
       <c r="C545" s="2" t="inlineStr"/>
       <c r="D545" s="2" t="inlineStr">
         <is>
-          <t>subscription_contract_renewal_terms AND rule_097_evidence -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
+          <t>subscription_contract_renewal_terms -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
         </is>
       </c>
       <c r="E545" s="2" t="inlineStr"/>
@@ -29366,7 +29418,7 @@
       <c r="C559" s="2" t="inlineStr"/>
       <c r="D559" s="2" t="inlineStr">
         <is>
-          <t>executive_sla_breach_terms AND rule_100_evidence -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
+          <t>executive_sla_breach_terms -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
         </is>
       </c>
       <c r="E559" s="2" t="inlineStr">
@@ -29426,7 +29478,7 @@
       <c r="C560" s="2" t="inlineStr"/>
       <c r="D560" s="2" t="inlineStr">
         <is>
-          <t>executive_sla_breach_terms AND rule_100_evidence -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
+          <t>executive_sla_breach_terms -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
         </is>
       </c>
       <c r="E560" s="2" t="inlineStr"/>
@@ -29480,7 +29532,7 @@
       <c r="C561" s="2" t="inlineStr"/>
       <c r="D561" s="2" t="inlineStr">
         <is>
-          <t>executive_sla_breach_terms AND rule_100_evidence -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
+          <t>executive_sla_breach_terms -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
         </is>
       </c>
       <c r="E561" s="2" t="inlineStr"/>
@@ -29524,7 +29576,7 @@
       <c r="C562" s="2" t="inlineStr"/>
       <c r="D562" s="2" t="inlineStr">
         <is>
-          <t>executive_sla_breach_terms AND rule_100_evidence -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
+          <t>executive_sla_breach_terms -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
         </is>
       </c>
       <c r="E562" s="2" t="inlineStr"/>
@@ -29568,7 +29620,7 @@
       <c r="C563" s="2" t="inlineStr"/>
       <c r="D563" s="2" t="inlineStr">
         <is>
-          <t>executive_sla_breach_terms AND rule_100_evidence -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
+          <t>executive_sla_breach_terms -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
         </is>
       </c>
       <c r="E563" s="2" t="inlineStr"/>
@@ -32487,14 +32539,22 @@
     <row r="620">
       <c r="A620" s="2" t="inlineStr">
         <is>
-          <t>RTE-0001</t>
-        </is>
-      </c>
-      <c r="B620" s="2" t="inlineStr"/>
-      <c r="C620" s="2" t="inlineStr"/>
+          <t>CFB-ACCOUNT</t>
+        </is>
+      </c>
+      <c r="B620" s="2" t="inlineStr">
+        <is>
+          <t>ACCOUNT</t>
+        </is>
+      </c>
+      <c r="C620" s="2" t="inlineStr">
+        <is>
+          <t>ACCOUNT_LOCKED</t>
+        </is>
+      </c>
       <c r="D620" s="2" t="inlineStr">
         <is>
-          <t>always (catch-all) -- Unrecognised complaint</t>
+          <t>account_terms -- Account problem, sub-type not stated</t>
         </is>
       </c>
       <c r="E620" s="2" t="inlineStr">
@@ -32504,12 +32564,12 @@
       </c>
       <c r="F620" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="G620" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H620" s="2" t="inlineStr"/>
@@ -32519,25 +32579,617 @@
       <c r="L620" s="2" t="inlineStr"/>
       <c r="M620" s="2" t="inlineStr">
         <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N620" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O620" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P620" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="inlineStr">
+        <is>
+          <t>CFB-BILLING</t>
+        </is>
+      </c>
+      <c r="B621" s="2" t="inlineStr">
+        <is>
+          <t>BILLING</t>
+        </is>
+      </c>
+      <c r="C621" s="2" t="inlineStr">
+        <is>
+          <t>INCORRECT_CHARGE</t>
+        </is>
+      </c>
+      <c r="D621" s="2" t="inlineStr">
+        <is>
+          <t>billing_error -- Disputed charge, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E621" s="2" t="inlineStr">
+        <is>
+          <t>BILLING</t>
+        </is>
+      </c>
+      <c r="F621" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G621" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H621" s="2" t="inlineStr"/>
+      <c r="I621" s="2" t="inlineStr"/>
+      <c r="J621" s="2" t="inlineStr"/>
+      <c r="K621" s="2" t="inlineStr"/>
+      <c r="L621" s="2" t="inlineStr"/>
+      <c r="M621" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N621" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O621" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P621" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="inlineStr">
+        <is>
+          <t>CFB-CUSTOMS</t>
+        </is>
+      </c>
+      <c r="B622" s="2" t="inlineStr">
+        <is>
+          <t>CUSTOMS</t>
+        </is>
+      </c>
+      <c r="C622" s="2" t="inlineStr">
+        <is>
+          <t>REGULATORY_IMPOUNDMENT_HOLD</t>
+        </is>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>customs_terms -- Customs or regulatory hold, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E622" s="2" t="inlineStr">
+        <is>
+          <t>COMPLIANCE</t>
+        </is>
+      </c>
+      <c r="F622" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G622" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H622" s="2" t="inlineStr"/>
+      <c r="I622" s="2" t="inlineStr"/>
+      <c r="J622" s="2" t="inlineStr"/>
+      <c r="K622" s="2" t="inlineStr"/>
+      <c r="L622" s="2" t="inlineStr"/>
+      <c r="M622" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N622" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O622" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P622" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="inlineStr">
+        <is>
+          <t>CFB-DELIVERY</t>
+        </is>
+      </c>
+      <c r="B623" s="2" t="inlineStr">
+        <is>
+          <t>DELIVERY</t>
+        </is>
+      </c>
+      <c r="C623" s="2" t="inlineStr">
+        <is>
+          <t>DELAYED_DELIVERY</t>
+        </is>
+      </c>
+      <c r="D623" s="2" t="inlineStr">
+        <is>
+          <t>delivery_failure OR delivery_delay OR delivery_inquiry_terms -- Delivery problem, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E623" s="2" t="inlineStr">
+        <is>
+          <t>LOGISTICS_OPS</t>
+        </is>
+      </c>
+      <c r="F623" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G623" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H623" s="2" t="inlineStr"/>
+      <c r="I623" s="2" t="inlineStr"/>
+      <c r="J623" s="2" t="inlineStr"/>
+      <c r="K623" s="2" t="inlineStr"/>
+      <c r="L623" s="2" t="inlineStr"/>
+      <c r="M623" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N623" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O623" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P623" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="inlineStr">
+        <is>
+          <t>CFB-PRODUCT-DEFECT</t>
+        </is>
+      </c>
+      <c r="B624" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DEFECT</t>
+        </is>
+      </c>
+      <c r="C624" s="2" t="inlineStr">
+        <is>
+          <t>DAMAGED_PARCEL</t>
+        </is>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>product_defect_terms -- Goods arrived damaged or faulty, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E624" s="2" t="inlineStr">
+        <is>
+          <t>WARRANTY_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F624" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G624" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H624" s="2" t="inlineStr"/>
+      <c r="I624" s="2" t="inlineStr"/>
+      <c r="J624" s="2" t="inlineStr"/>
+      <c r="K624" s="2" t="inlineStr"/>
+      <c r="L624" s="2" t="inlineStr"/>
+      <c r="M624" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N624" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O624" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P624" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="inlineStr">
+        <is>
+          <t>CFB-REFUND</t>
+        </is>
+      </c>
+      <c r="B625" s="2" t="inlineStr">
+        <is>
+          <t>REFUND</t>
+        </is>
+      </c>
+      <c r="C625" s="2" t="inlineStr">
+        <is>
+          <t>REFUND_NOT_PROCESSED</t>
+        </is>
+      </c>
+      <c r="D625" s="2" t="inlineStr">
+        <is>
+          <t>refund_terms OR refund_failure -- Refund request, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E625" s="2" t="inlineStr">
+        <is>
+          <t>RETURNS_REFUNDS; support: BILLING</t>
+        </is>
+      </c>
+      <c r="F625" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G625" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H625" s="2" t="inlineStr"/>
+      <c r="I625" s="2" t="inlineStr"/>
+      <c r="J625" s="2" t="inlineStr"/>
+      <c r="K625" s="2" t="inlineStr"/>
+      <c r="L625" s="2" t="inlineStr"/>
+      <c r="M625" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N625" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O625" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P625" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="inlineStr">
+        <is>
+          <t>CFB-SAFETY</t>
+        </is>
+      </c>
+      <c r="B626" s="2" t="inlineStr">
+        <is>
+          <t>SAFETY</t>
+        </is>
+      </c>
+      <c r="C626" s="2" t="inlineStr">
+        <is>
+          <t>RECKLESS_DRIVING_SAFETY_RISK</t>
+        </is>
+      </c>
+      <c r="D626" s="2" t="inlineStr">
+        <is>
+          <t>safety_lexicon_hit OR injury_mention -- Safety incident, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E626" s="2" t="inlineStr">
+        <is>
+          <t>SAFETY; support: LOGISTICS_OPS</t>
+        </is>
+      </c>
+      <c r="F626" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G626" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H626" s="2" t="inlineStr"/>
+      <c r="I626" s="2" t="inlineStr"/>
+      <c r="J626" s="2" t="inlineStr"/>
+      <c r="K626" s="2" t="inlineStr"/>
+      <c r="L626" s="2" t="inlineStr"/>
+      <c r="M626" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N626" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O626" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P626" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="inlineStr">
+        <is>
+          <t>CFB-STAFF</t>
+        </is>
+      </c>
+      <c r="B627" s="2" t="inlineStr">
+        <is>
+          <t>STAFF_BEHAVIOR</t>
+        </is>
+      </c>
+      <c r="C627" s="2" t="inlineStr">
+        <is>
+          <t>RUDE_RIDER_DRIVER_BEHAVIOR</t>
+        </is>
+      </c>
+      <c r="D627" s="2" t="inlineStr">
+        <is>
+          <t>staff_conduct_terms -- Staff conduct, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E627" s="2" t="inlineStr">
+        <is>
+          <t>LOGISTICS_OPS; support: CUSTOMER_RELATIONS</t>
+        </is>
+      </c>
+      <c r="F627" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G627" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H627" s="2" t="inlineStr"/>
+      <c r="I627" s="2" t="inlineStr"/>
+      <c r="J627" s="2" t="inlineStr"/>
+      <c r="K627" s="2" t="inlineStr"/>
+      <c r="L627" s="2" t="inlineStr"/>
+      <c r="M627" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N627" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O627" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P627" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="inlineStr">
+        <is>
+          <t>CFB-TECHNICAL</t>
+        </is>
+      </c>
+      <c r="B628" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL_SUPPORT</t>
+        </is>
+      </c>
+      <c r="C628" s="2" t="inlineStr">
+        <is>
+          <t>APP_CRASH</t>
+        </is>
+      </c>
+      <c r="D628" s="2" t="inlineStr">
+        <is>
+          <t>technical_terms -- App or portal problem, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E628" s="2" t="inlineStr">
+        <is>
+          <t>CUSTOMER_RELATIONS</t>
+        </is>
+      </c>
+      <c r="F628" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G628" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H628" s="2" t="inlineStr"/>
+      <c r="I628" s="2" t="inlineStr"/>
+      <c r="J628" s="2" t="inlineStr"/>
+      <c r="K628" s="2" t="inlineStr"/>
+      <c r="L628" s="2" t="inlineStr"/>
+      <c r="M628" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N628" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O628" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P628" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="inlineStr">
+        <is>
+          <t>CFB-WARRANTY</t>
+        </is>
+      </c>
+      <c r="B629" s="2" t="inlineStr">
+        <is>
+          <t>WARRANTY</t>
+        </is>
+      </c>
+      <c r="C629" s="2" t="inlineStr">
+        <is>
+          <t>WARRANTY_CLAIM_DENIED</t>
+        </is>
+      </c>
+      <c r="D629" s="2" t="inlineStr">
+        <is>
+          <t>warranty_terms -- Warranty or claim, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E629" s="2" t="inlineStr">
+        <is>
+          <t>WARRANTY_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F629" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G629" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H629" s="2" t="inlineStr"/>
+      <c r="I629" s="2" t="inlineStr"/>
+      <c r="J629" s="2" t="inlineStr"/>
+      <c r="K629" s="2" t="inlineStr"/>
+      <c r="L629" s="2" t="inlineStr"/>
+      <c r="M629" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N629" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O629" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P629" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="inlineStr">
+        <is>
+          <t>RTE-0001</t>
+        </is>
+      </c>
+      <c r="B630" s="2" t="inlineStr"/>
+      <c r="C630" s="2" t="inlineStr"/>
+      <c r="D630" s="2" t="inlineStr">
+        <is>
+          <t>always (catch-all) -- Unrecognised complaint</t>
+        </is>
+      </c>
+      <c r="E630" s="2" t="inlineStr">
+        <is>
+          <t>CUSTOMER_RELATIONS</t>
+        </is>
+      </c>
+      <c r="F630" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G630" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H630" s="2" t="inlineStr"/>
+      <c r="I630" s="2" t="inlineStr"/>
+      <c r="J630" s="2" t="inlineStr"/>
+      <c r="K630" s="2" t="inlineStr"/>
+      <c r="L630" s="2" t="inlineStr"/>
+      <c r="M630" s="2" t="inlineStr">
+        <is>
           <t>ROUTING</t>
         </is>
       </c>
-      <c r="N620" s="2" t="n">
+      <c r="N630" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="O620" s="2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="P620" s="2" t="inlineStr">
+      <c r="O630" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P630" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P620"/>
+  <autoFilter ref="A1:P630"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -32548,7 +33200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P117"/>
+  <dimension ref="A1:P127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -32669,7 +33321,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>RULE-001: delayed_delivery_terms; RES-001, ELG-001-COMP, ELG-001-REFU, ELG-001-REPL: delayed_delivery_terms AND rule_001_evidence -- Standard domestic transit delay under 24 hours without perishable contents</t>
+          <t>delayed_delivery_terms -- Standard domestic transit delay under 24 hours without perishable contents</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -32914,7 +33566,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>RULE-004: missed_delivery_attempt_terms; RES-004, ELG-004-COMP, ELG-004-REFU, ELG-004-REPL: missed_delivery_attempt_terms AND rule_004_evidence -- First missed delivery attempt due to customer premises locked or phone unattended</t>
+          <t>missed_delivery_attempt_terms -- First missed delivery attempt due to customer premises locked or phone unattended</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -33095,7 +33747,11 @@
           <t>DOC-003-S4 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: REQUIRES_VERIFICATION (human approval); Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
           <t>Move parcel to 48-hour hub retention bay
@@ -33151,7 +33807,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>RULE-007: package_left_unattended_terms; RES-007, ELG-007-COMP, ELG-007-REFU, ELG-007-REPL: package_left_unattended_terms AND rule_007_evidence -- Package left on porch or with building guard with prior verbal consignee permission</t>
+          <t>package_left_unattended_terms -- Package left on porch or with building guard with prior verbal consignee permission</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -33247,7 +33903,11 @@
           <t>DOC-003-S3 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: NOT_ELIGIBLE; Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
           <t>Issue written compliance warning to courier
@@ -33382,7 +34042,7 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>RULE-010: wrong_route_dispatch_terms; RES-010, ELG-010-COMP, ELG-010-REFU, ELG-010-REPL: wrong_route_dispatch_terms AND rule_010_evidence -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan)</t>
+          <t>wrong_route_dispatch_terms -- Parcel misrouted to incorrect local branch within same city (e.g. Clifton instead of Gulshan)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -33649,7 +34309,11 @@
           <t>DOC-007-S1 | Eligibility - Compensation: ELIGIBLE; Refund: ELIGIBLE; Replacement: ELIGIBLE</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
           <t>Trigger 48-hour all-hub physical inventory search
@@ -33705,7 +34369,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>RULE-014: lost_parcel_terms; ESC-014, RES-014, ELG-014-COMP, ELG-014-REFU, ELG-014-REPL: lost_parcel_terms AND rule_014_evidence -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
+          <t>lost_parcel_terms -- Insured shipment lost in transit with declared value between PKR 15,000 and PKR 100,000</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -33894,7 +34558,11 @@
           <t>DOC-007-S2 | Eligibility - Compensation: REQUIRES_VERIFICATION (human approval); Refund: REQUIRES_VERIFICATION (human approval); Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
           <t>Locate missing box piece-identifier barcode across transit nodes
@@ -33950,7 +34618,7 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>RULE-017: partial_shipment_missing_terms; ESC-017, RES-017, ELG-017-COMP, ELG-017-REFU, ELG-017-REPL: partial_shipment_missing_terms AND rule_017_evidence -- Partial loss confirmed stolen from damaged outer master carton</t>
+          <t>partial_shipment_missing_terms -- Partial loss confirmed stolen from damaged outer master carton</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -34115,7 +34783,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>RULE-019: damaged_parcel_terms; RES-019, ELG-019-COMP, ELG-019-REFU, ELG-019-REPL: damaged_parcel_terms AND rule_019_evidence -- Minor outer carton denting with internal goods completely undamaged</t>
+          <t>damaged_parcel_terms -- Minor outer carton denting with internal goods completely undamaged</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -34212,7 +34880,11 @@
           <t>DOC-007-S2 | Eligibility - Compensation: ELIGIBLE; Refund: ELIGIBLE; Replacement: ELIGIBLE</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
           <t>Verify Fragile label was affixed at origin booking
@@ -34434,7 +35106,7 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>RULE-023: wrong_item_delivered_terms; RES-023, ELG-023-COMP, ELG-023-REFU, ELG-023-REPL: wrong_item_delivered_terms AND rule_023_evidence -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
+          <t>wrong_item_delivered_terms -- Merchant packed wrong SKU / manifest matches parcel contents but merchant made error</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -34592,7 +35264,7 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>RULE-025: tampered_packaging_terms; RES-025, ELG-025-COMP, ELG-025-REFU, ELG-025-REPL: tampered_packaging_terms AND rule_025_evidence -- Parcel received with broken security tape but all items accounted for and intact</t>
+          <t>tampered_packaging_terms -- Parcel received with broken security tape but all items accounted for and intact</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -34615,7 +35287,11 @@
           <t>DOC-009-S3 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: NOT_ELIGIBLE; Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
           <t>Log security tape breach in hub quality audit log
@@ -34914,7 +35590,7 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>RULE-029: cod_amount_mismatch_terms; RES-029, ELG-029-COMP, ELG-029-REFU, ELG-029-REPL: cod_amount_mismatch_terms AND rule_029_evidence -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
+          <t>cod_amount_mismatch_terms -- Merchant booked wrong COD amount on portal and requests in-transit correction</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
@@ -35072,7 +35748,7 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>RULE-031: duplicate_charge_terms; RES-031, ELG-031-COMP, ELG-031-REFU, ELG-031-REPL: duplicate_charge_terms AND rule_031_evidence -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
+          <t>duplicate_charge_terms -- Customer online portal shows two identical invoice charges for a single consignment booking</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -35315,7 +35991,7 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>RULE-034: incorrect_charge_terms; RES-034, ELG-034-COMP, ELG-034-REFU, ELG-034-REPL: incorrect_charge_terms AND rule_034_evidence -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,000)</t>
+          <t>incorrect_charge_terms -- Dispute over volumetric vs dead weight calculation resulting in minor overcharge (&lt; PKR 1,000)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -35553,7 +36229,7 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>RULE-037: cod_remittance_delay_terms; RES-037, ELG-037-COMP, ELG-037-REFU, ELG-037-REPL: cod_remittance_delay_terms AND rule_037_evidence -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
+          <t>cod_remittance_delay_terms -- Merchant COD remittance delayed past standard Wednesday cycle due to bank holiday</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
@@ -35792,7 +36468,7 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>RULE-040: refund_not_processed_terms; RES-040, ELG-040-COMP, ELG-040-REFU, ELG-040-REPL: refund_not_processed_terms AND rule_040_evidence -- Customer refund requested within 7-day policy window, all documentation verified</t>
+          <t>refund_not_processed_terms -- Customer refund requested within 7-day policy window, all documentation verified</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -36037,7 +36713,7 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>RULE-043: refund_delay_terms; RES-043, ELG-043-COMP, ELG-043-REFU, ELG-043-REPL: refund_delay_terms AND rule_043_evidence -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
+          <t>refund_delay_terms -- Customer inquiry regarding refund status currently on day 3 of 5-7 day standard SLA</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
@@ -36271,7 +36947,7 @@
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>RULE-046: rto_processing_delay_terms; RES-046, ELG-046-COMP, ELG-046-REFU, ELG-046-REPL: rto_processing_delay_terms AND rule_046_evidence -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
+          <t>rto_processing_delay_terms -- Failed delivery consignment held in hub awaiting scheduled weekly RTO consolidation</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
@@ -36509,7 +37185,7 @@
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>RULE-049: account_locked_terms; RES-049, ELG-049-COMP, ELG-049-REFU, ELG-049-REPL: account_locked_terms AND rule_049_evidence -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
+          <t>account_locked_terms -- Consumer portal account locked after 5 consecutive incorrect password attempts</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
@@ -36748,7 +37424,7 @@
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>RULE-052: unauthorized_account_access_terms; ESC-052, RES-052, ELG-052-COMP, ELG-052-REFU, ELG-052-REPL: unauthorized_account_access_terms AND rule_052_evidence -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
+          <t>unauthorized_account_access_terms -- Customer reports suspicious login alert from unfamiliar city/IP address, no funds diverted</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
@@ -36995,7 +37671,7 @@
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>RULE-055: merchant_profile_update_terms; RES-055, ELG-055-COMP, ELG-055-REFU, ELG-055-REPL: merchant_profile_update_terms AND rule_055_evidence -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
+          <t>merchant_profile_update_terms -- Merchant requests standard update to pickup warehouse address or contact phone number</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
@@ -37092,7 +37768,11 @@
           <t>DOC-021-S1 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: NOT_ELIGIBLE; Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>COMPLIANCE_REVIEW</t>
+        </is>
+      </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
           <t>Collect updated FBR NTN certificate and SECP incorporation form
@@ -37230,7 +37910,7 @@
       </c>
       <c r="D59" s="2" t="inlineStr">
         <is>
-          <t>RULE-058: tracking_not_updating_terms; RES-058, ELG-058-COMP, ELG-058-REFU, ELG-058-REPL: tracking_not_updating_terms AND rule_058_evidence -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
+          <t>tracking_not_updating_terms -- Consignment tracking scan stationary for 12 hours during overnight inter-city linehaul</t>
         </is>
       </c>
       <c r="E59" s="2" t="inlineStr">
@@ -37468,7 +38148,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>RULE-061: app_crash_terms; RES-061, ELG-061-COMP, ELG-061-REFU, ELG-061-REPL: app_crash_terms AND rule_061_evidence -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
+          <t>app_crash_terms -- Single user reports mobile tracking app crashes on specific older Android OS version</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -37647,7 +38327,11 @@
           <t>DOC-023-S2 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: NOT_ELIGIBLE; Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
           <t>Provide merchant temporary split-CSV upload workaround
@@ -37702,7 +38386,7 @@
       </c>
       <c r="D65" s="2" t="inlineStr">
         <is>
-          <t>RULE-064: api_webhook_failure_terms; RES-064, ELG-064-COMP, ELG-064-REFU, ELG-064-REPL: api_webhook_failure_terms AND rule_064_evidence -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
+          <t>api_webhook_failure_terms -- Merchant reports webhook delivery notification latency of 15 minutes during peak hours</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -37799,7 +38483,11 @@
           <t>DOC-023-S2 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: NOT_ELIGIBLE; Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I66" s="2" t="inlineStr"/>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
           <t>Verify SSL handshake logs from outbound webhook gateway
@@ -37936,7 +38624,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>RULE-067: rude_rider_driver_behavior_terms; RES-067, ELG-067-COMP, ELG-067-REFU, ELG-067-REPL: rude_rider_driver_behavior_terms AND rule_067_evidence -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
+          <t>rude_rider_driver_behavior_terms -- Customer reports rider spoke discourteously or showed impatient attitude during delivery</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -37959,7 +38647,11 @@
           <t>DOC-020-S1 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: NOT_ELIGIBLE; Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
           <t>Call customer to convey formal company apology
@@ -38180,7 +38872,7 @@
       </c>
       <c r="D71" s="2" t="inlineStr">
         <is>
-          <t>RULE-070: rider_demanding_cash_tip_terms; RES-070, ELG-070-COMP, ELG-070-REFU, ELG-070-REPL: rider_demanding_cash_tip_terms AND rule_070_evidence -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and received parcel</t>
+          <t>rider_demanding_cash_tip_terms -- Rider verbally asks for tip / round-up change on prepaid shipment, customer refused and received parcel</t>
         </is>
       </c>
       <c r="E71" s="2" t="inlineStr">
@@ -38203,7 +38895,11 @@
           <t>DOC-021-S2 | Eligibility - Compensation: REQUIRES_VERIFICATION (human approval); Refund: NOT_ELIGIBLE; Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>SUPERVISOR</t>
+        </is>
+      </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
           <t>Interview rider and reiterate strict zero-solicitation policy
@@ -38419,7 +39115,7 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>RULE-073: warranty_claim_denied_terms; RES-073, ELG-073-COMP, ELG-073-REFU, ELG-073-REPL: warranty_claim_denied_terms AND rule_073_evidence -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
+          <t>warranty_claim_denied_terms -- Customer disputes warranty claim denial on non-insured cargo damaged by improper packaging</t>
         </is>
       </c>
       <c r="E74" s="2" t="inlineStr">
@@ -38658,7 +39354,7 @@
       </c>
       <c r="D77" s="2" t="inlineStr">
         <is>
-          <t>RULE-076: insurance_payout_delay_terms; RES-076, ELG-076-COMP, ELG-076-REFU, ELG-076-REPL: insurance_payout_delay_terms AND rule_076_evidence -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
+          <t>insurance_payout_delay_terms -- Customer insurance claim approved, awaiting standard 21-day insurer settlement cycle</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
@@ -38895,7 +39591,7 @@
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>RULE-079: data_privacy_breach_terms; ESC-079, RES-079, ELG-079-COMP, ELG-079-REFU, ELG-079-REPL: data_privacy_breach_terms AND rule_079_evidence -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
+          <t>data_privacy_breach_terms -- Customer reports courier sent unsolicited personal message on WhatsApp after delivery</t>
         </is>
       </c>
       <c r="E80" s="2" t="inlineStr">
@@ -39084,7 +39780,11 @@
           <t>DOC-015-S3 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: NOT_ELIGIBLE; Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr"/>
+      <c r="I82" s="2" t="inlineStr">
+        <is>
+          <t>COMPLIANCE_REVIEW</t>
+        </is>
+      </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
           <t>Verify requester identity and CNIC credentials
@@ -39135,7 +39835,7 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>RULE-082: unsolicited_marketing_sms_terms; RES-082, ELG-082-COMP, ELG-082-REFU, ELG-082-REPL: unsolicited_marketing_sms_terms AND rule_082_evidence -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
+          <t>unsolicited_marketing_sms_terms -- Customer requests opt-out from promotional broadcast SMS marketing campaigns</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
@@ -39372,7 +40072,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>RULE-085: reckless_driving_safety_risk_terms; ESC-085, RES-085, ELG-085-COMP, ELG-085-REFU, ELG-085-REPL: reckless_driving_safety_risk_terms AND rule_085_evidence -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
+          <t>reckless_driving_safety_risk_terms -- Citizen reports courier van driving recklessly / speeding in residential neighborhood</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -39616,7 +40316,7 @@
       </c>
       <c r="D89" s="2" t="inlineStr">
         <is>
-          <t>RULE-088: hazardous_material_mishandling_terms; RES-088, ELG-088-COMP, ELG-088-REFU, ELG-088-REPL: hazardous_material_mishandling_terms AND rule_088_evidence -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
+          <t>hazardous_material_mishandling_terms -- Hub staff identifies parcel emitting pungent odor / small non-toxic cosmetic liquid leak</t>
         </is>
       </c>
       <c r="E89" s="2" t="inlineStr">
@@ -39639,7 +40339,11 @@
           <t>DOC-025-S2 | Eligibility - Compensation: NOT_ELIGIBLE; Refund: REQUIRES_VERIFICATION (human approval); Replacement: NOT_ELIGIBLE</t>
         </is>
       </c>
-      <c r="I89" s="2" t="inlineStr"/>
+      <c r="I89" s="2" t="inlineStr">
+        <is>
+          <t>SPECIALIST</t>
+        </is>
+      </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
           <t>Isolate parcel in ventilated hub containment bay
@@ -39860,7 +40564,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>RULE-091: missing_customs_documents_terms; RES-091, ELG-091-COMP, ELG-091-REFU, ELG-091-REPL: missing_customs_documents_terms AND rule_091_evidence -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on file</t>
+          <t>missing_customs_documents_terms -- Inter-provincial consignment missing commercial invoice copy in outer pouch; digital copy on file</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -40099,7 +40803,7 @@
       </c>
       <c r="D95" s="2" t="inlineStr">
         <is>
-          <t>RULE-094: regulatory_impoundment_hold_terms; RES-094, ELG-094-COMP, ELG-094-REFU, ELG-094-REPL: regulatory_impoundment_hold_terms AND rule_094_evidence -- Consignment held for routine random provincial excise vehicle weight and document check</t>
+          <t>regulatory_impoundment_hold_terms -- Consignment held for routine random provincial excise vehicle weight and document check</t>
         </is>
       </c>
       <c r="E95" s="2" t="inlineStr">
@@ -40337,7 +41041,7 @@
       </c>
       <c r="D98" s="2" t="inlineStr">
         <is>
-          <t>RULE-097: subscription_contract_renewal_terms; RES-097, ELG-097-COMP, ELG-097-REFU, ELG-097-REPL: subscription_contract_renewal_terms AND rule_097_evidence -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
+          <t>subscription_contract_renewal_terms -- Corporate freight client requests routine annual rate review and SLA contract renewal</t>
         </is>
       </c>
       <c r="E98" s="2" t="inlineStr">
@@ -40575,7 +41279,7 @@
       </c>
       <c r="D101" s="2" t="inlineStr">
         <is>
-          <t>RULE-100: executive_sla_breach_terms; ESC-100, RES-100, ELG-100-COMP, ELG-100-REFU, ELG-100-REPL: executive_sla_breach_terms AND rule_100_evidence -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
+          <t>executive_sla_breach_terms -- VIP consumer shipment misses guaranteed overnight delivery commitment by 4 hours</t>
         </is>
       </c>
       <c r="E101" s="2" t="inlineStr">
@@ -41692,14 +42396,22 @@
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>RTE-0001</t>
-        </is>
-      </c>
-      <c r="B117" s="2" t="inlineStr"/>
-      <c r="C117" s="2" t="inlineStr"/>
+          <t>CFB-ACCOUNT</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>ACCOUNT</t>
+        </is>
+      </c>
+      <c r="C117" s="2" t="inlineStr">
+        <is>
+          <t>ACCOUNT_LOCKED</t>
+        </is>
+      </c>
       <c r="D117" s="2" t="inlineStr">
         <is>
-          <t>always (catch-all) -- Unrecognised complaint</t>
+          <t>account_terms -- Account problem, sub-type not stated</t>
         </is>
       </c>
       <c r="E117" s="2" t="inlineStr">
@@ -41709,12 +42421,12 @@
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr"/>
@@ -41724,25 +42436,617 @@
       <c r="L117" s="2" t="inlineStr"/>
       <c r="M117" s="2" t="inlineStr">
         <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N117" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P117" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>CFB-BILLING</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>BILLING</t>
+        </is>
+      </c>
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>INCORRECT_CHARGE</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>billing_error -- Disputed charge, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>BILLING</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr"/>
+      <c r="I118" s="2" t="inlineStr"/>
+      <c r="J118" s="2" t="inlineStr"/>
+      <c r="K118" s="2" t="inlineStr"/>
+      <c r="L118" s="2" t="inlineStr"/>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O118" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P118" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>CFB-CUSTOMS</t>
+        </is>
+      </c>
+      <c r="B119" s="2" t="inlineStr">
+        <is>
+          <t>CUSTOMS</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="inlineStr">
+        <is>
+          <t>REGULATORY_IMPOUNDMENT_HOLD</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>customs_terms -- Customs or regulatory hold, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E119" s="2" t="inlineStr">
+        <is>
+          <t>COMPLIANCE</t>
+        </is>
+      </c>
+      <c r="F119" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G119" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H119" s="2" t="inlineStr"/>
+      <c r="I119" s="2" t="inlineStr"/>
+      <c r="J119" s="2" t="inlineStr"/>
+      <c r="K119" s="2" t="inlineStr"/>
+      <c r="L119" s="2" t="inlineStr"/>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N119" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P119" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>CFB-DELIVERY</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>DELIVERY</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>DELAYED_DELIVERY</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>delivery_failure OR delivery_delay OR delivery_inquiry_terms -- Delivery problem, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
+        <is>
+          <t>LOGISTICS_OPS</t>
+        </is>
+      </c>
+      <c r="F120" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr"/>
+      <c r="I120" s="2" t="inlineStr"/>
+      <c r="J120" s="2" t="inlineStr"/>
+      <c r="K120" s="2" t="inlineStr"/>
+      <c r="L120" s="2" t="inlineStr"/>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N120" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P120" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>CFB-PRODUCT-DEFECT</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>PRODUCT_DEFECT</t>
+        </is>
+      </c>
+      <c r="C121" s="2" t="inlineStr">
+        <is>
+          <t>DAMAGED_PARCEL</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>product_defect_terms -- Goods arrived damaged or faulty, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E121" s="2" t="inlineStr">
+        <is>
+          <t>WARRANTY_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F121" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G121" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H121" s="2" t="inlineStr"/>
+      <c r="I121" s="2" t="inlineStr"/>
+      <c r="J121" s="2" t="inlineStr"/>
+      <c r="K121" s="2" t="inlineStr"/>
+      <c r="L121" s="2" t="inlineStr"/>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N121" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O121" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P121" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>CFB-REFUND</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>REFUND</t>
+        </is>
+      </c>
+      <c r="C122" s="2" t="inlineStr">
+        <is>
+          <t>REFUND_NOT_PROCESSED</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>refund_terms OR refund_failure -- Refund request, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E122" s="2" t="inlineStr">
+        <is>
+          <t>RETURNS_REFUNDS; support: BILLING</t>
+        </is>
+      </c>
+      <c r="F122" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G122" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H122" s="2" t="inlineStr"/>
+      <c r="I122" s="2" t="inlineStr"/>
+      <c r="J122" s="2" t="inlineStr"/>
+      <c r="K122" s="2" t="inlineStr"/>
+      <c r="L122" s="2" t="inlineStr"/>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N122" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O122" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P122" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>CFB-SAFETY</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>SAFETY</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>RECKLESS_DRIVING_SAFETY_RISK</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>safety_lexicon_hit OR injury_mention -- Safety incident, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E123" s="2" t="inlineStr">
+        <is>
+          <t>SAFETY; support: LOGISTICS_OPS</t>
+        </is>
+      </c>
+      <c r="F123" s="2" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr"/>
+      <c r="I123" s="2" t="inlineStr"/>
+      <c r="J123" s="2" t="inlineStr"/>
+      <c r="K123" s="2" t="inlineStr"/>
+      <c r="L123" s="2" t="inlineStr"/>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N123" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O123" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P123" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>CFB-STAFF</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>STAFF_BEHAVIOR</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>RUDE_RIDER_DRIVER_BEHAVIOR</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>staff_conduct_terms -- Staff conduct, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>LOGISTICS_OPS; support: CUSTOMER_RELATIONS</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr"/>
+      <c r="I124" s="2" t="inlineStr"/>
+      <c r="J124" s="2" t="inlineStr"/>
+      <c r="K124" s="2" t="inlineStr"/>
+      <c r="L124" s="2" t="inlineStr"/>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N124" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P124" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>CFB-TECHNICAL</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>TECHNICAL_SUPPORT</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>APP_CRASH</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>technical_terms -- App or portal problem, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>CUSTOMER_RELATIONS</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr"/>
+      <c r="I125" s="2" t="inlineStr"/>
+      <c r="J125" s="2" t="inlineStr"/>
+      <c r="K125" s="2" t="inlineStr"/>
+      <c r="L125" s="2" t="inlineStr"/>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N125" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P125" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>CFB-WARRANTY</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>WARRANTY</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>WARRANTY_CLAIM_DENIED</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>warranty_terms -- Warranty or claim, sub-type not stated</t>
+        </is>
+      </c>
+      <c r="E126" s="2" t="inlineStr">
+        <is>
+          <t>WARRANTY_CLAIMS</t>
+        </is>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr"/>
+      <c r="I126" s="2" t="inlineStr"/>
+      <c r="J126" s="2" t="inlineStr"/>
+      <c r="K126" s="2" t="inlineStr"/>
+      <c r="L126" s="2" t="inlineStr"/>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>CLASSIFICATION</t>
+        </is>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P126" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>RTE-0001</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr"/>
+      <c r="C127" s="2" t="inlineStr"/>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>always (catch-all) -- Unrecognised complaint</t>
+        </is>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>CUSTOMER_RELATIONS</t>
+        </is>
+      </c>
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="H127" s="2" t="inlineStr"/>
+      <c r="I127" s="2" t="inlineStr"/>
+      <c r="J127" s="2" t="inlineStr"/>
+      <c r="K127" s="2" t="inlineStr"/>
+      <c r="L127" s="2" t="inlineStr"/>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
           <t>ROUTING</t>
         </is>
       </c>
-      <c r="N117" s="2" t="n">
+      <c r="N127" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="O117" s="2" t="inlineStr">
-        <is>
-          <t>1.0</t>
-        </is>
-      </c>
-      <c r="P117" s="2" t="inlineStr">
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="P127" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P117"/>
+  <autoFilter ref="A1:P127"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -41753,7 +43057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -41776,7 +43080,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-27 15:02</t>
+          <t>2026-09-28 07:09</t>
         </is>
       </c>
     </row>
@@ -41800,7 +43104,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>004880e57af6f411250d16cd09d52a99a303dd7999102e859545bcb7dc8f6f61</t>
+          <t>3d964c97e6c8d9b42d260f82e545f8d3c903af11c6547faa61fc640a5e60596f</t>
         </is>
       </c>
     </row>
@@ -41812,7 +43116,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>004880e5</t>
+          <t>3d964c97</t>
         </is>
       </c>
     </row>
@@ -41835,7 +43139,7 @@
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>619</v>
+        <v>629</v>
       </c>
     </row>
     <row r="9">
@@ -41845,7 +43149,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>619</v>
+        <v>629</v>
       </c>
     </row>
     <row r="10">
@@ -41865,7 +43169,7 @@
         </is>
       </c>
       <c r="B11" s="2" t="n">
-        <v>107</v>
+        <v>117</v>
       </c>
     </row>
     <row r="12">
@@ -41925,7 +43229,7 @@
         </is>
       </c>
       <c r="B17" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18">
@@ -41945,7 +43249,7 @@
         </is>
       </c>
       <c r="B19" s="2" t="n">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20">
@@ -41965,7 +43269,7 @@
         </is>
       </c>
       <c r="B21" s="2" t="n">
-        <v>144</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22">
@@ -41995,166 +43299,178 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  complaint_rules/classification.yaml</t>
+          <t xml:space="preserve">  complaint_rules/category_fallback.yaml</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>ruleset=classification version=1.0 rules=107 sha256=d38a3a46322f</t>
+          <t>ruleset=category_fallback version=1.0 rules=10 sha256=d350256ba8a2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  complaint_rules/eligibility.yaml</t>
+          <t xml:space="preserve">  complaint_rules/classification.yaml</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>ruleset=eligibility version=1.0 rules=322 sha256=64bdcdca248c</t>
+          <t>ruleset=classification version=1.0 rules=107 sha256=04bca2bca39e</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  complaint_rules/resolution.yaml</t>
+          <t xml:space="preserve">  complaint_rules/eligibility.yaml</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>ruleset=resolution version=1.0 rules=115 sha256=c58172facb5b</t>
+          <t>ruleset=eligibility version=1.0 rules=322 sha256=f029f3c4fdde</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  routing_rules/departments.yaml</t>
+          <t xml:space="preserve">  complaint_rules/resolution.yaml</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>ruleset=routing version=1.0 rules=1 sha256=184f710bbf73</t>
+          <t>ruleset=resolution version=1.0 rules=115 sha256=be39c2184223</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">  routing_rules/departments.yaml</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>ruleset=routing version=1.0 rules=1 sha256=184f710bbf73</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">  escalation_rules/mandatory.yaml</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>ruleset=escalation version=1.0 rules=74 sha256=6fe098225243</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr"/>
-      <c r="B30" s="2" t="inlineStr"/>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>ruleset=escalation version=1.0 rules=74 sha256=822223cc642c</t>
+        </is>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr"/>
+      <c r="B31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Column notes</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Conditions</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Rendered 'when' tree, then '--' and the authored prose the rule is named after.</t>
-        </is>
-      </c>
+      <c r="B32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Department</t>
+          <t>Conditions</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Owning department; a supporting department is shown as 'support: CODE'.</t>
+          <t>Rendered 'when' tree, then '--' and the authored prose the rule is named after.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>Policy</t>
+          <t>Department</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Cited sections as DOC-nnn-Sn. For ELIGIBILITY rules also the entitlement verdict.</t>
+          <t>Owning department; a supporting department is shown as 'support: CODE'.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>Escalation</t>
+          <t>Policy</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>'(mandatory floor)' marks a level the engine may raise but never lower.</t>
+          <t>Cited sections as DOC-nnn-Sn. For ELIGIBILITY rules also the entitlement verdict.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>Follow-up</t>
+          <t>Escalation</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Yes where the YAML sets follow_up_required (or follow_up) to true; blank otherwise.</t>
+          <t>'(mandatory floor)' marks a level the engine may raise but never lower.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Follow-up</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>The 'version' field of the YAML file the rule is authored in.</t>
+          <t>Yes where the YAML sets follow_up_required (or follow_up) to true; blank otherwise.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>Blank cells</t>
+          <t>Version</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>The rule does not set that field. Nothing is filled in from another rule on the Rule Matrix sheet.</t>
+          <t>The 'version' field of the YAML file the rule is authored in.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
+          <t>Blank cells</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>The rule does not set that field. Nothing is filled in from another rule on the Rule Matrix sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
           <t>By Case</t>
         </is>
       </c>
-      <c r="B39" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>Rules of one lineage merged with the engine's semantics: highest precedence wins scalars, actions unioned, floor applied.</t>
         </is>

</xml_diff>